<commit_message>
refactor: remove legacy voting forms and update primary form versions
</commit_message>
<xml_diff>
--- a/All_Voting_Form_Repeat_V1.xlsx
+++ b/All_Voting_Form_Repeat_V1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Desktop\SurveyCTO_Voting_EVM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCEF8DB3-AAB3-4FF2-B0A3-E9135D2E577D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4127CA3E-5E8F-4084-82E1-65AA3EE0710A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,10 +17,6 @@
     <sheet name="choices" sheetId="2" r:id="rId2"/>
     <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">choices!$A$1:$G$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">survey!$A$1:$K$22</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,14 +33,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="234">
+  <si>
+    <t>name</t>
+  </si>
   <si>
     <t>type</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
     <t>label::English (en)</t>
   </si>
   <si>
@@ -87,12 +83,12 @@
     <t>phonenumber</t>
   </si>
   <si>
+    <t>device_info</t>
+  </si>
+  <si>
     <t>calculate</t>
   </si>
   <si>
-    <t>device_info</t>
-  </si>
-  <si>
     <t>false</t>
   </si>
   <si>
@@ -105,12 +101,12 @@
     <t>duration()</t>
   </si>
   <si>
+    <t>state</t>
+  </si>
+  <si>
     <t>select_one state_list</t>
   </si>
   <si>
-    <t>state</t>
-  </si>
-  <si>
     <t>State</t>
   </si>
   <si>
@@ -120,12 +116,12 @@
     <t>true</t>
   </si>
   <si>
+    <t>district</t>
+  </si>
+  <si>
     <t>select_one district_list</t>
   </si>
   <si>
-    <t>district</t>
-  </si>
-  <si>
     <t>District</t>
   </si>
   <si>
@@ -135,12 +131,12 @@
     <t>filter = ${state}</t>
   </si>
   <si>
+    <t>constituency</t>
+  </si>
+  <si>
     <t>select_one constituency_list</t>
   </si>
   <si>
-    <t>constituency</t>
-  </si>
-  <si>
     <t>Constituency</t>
   </si>
   <si>
@@ -150,60 +146,60 @@
     <t>filter = ${district}</t>
   </si>
   <si>
+    <t>village_name</t>
+  </si>
+  <si>
     <t>text</t>
   </si>
   <si>
-    <t>village_name</t>
-  </si>
-  <si>
     <t>Village Name</t>
   </si>
   <si>
     <t>गांव का नाम</t>
   </si>
   <si>
+    <t>voter_repeat</t>
+  </si>
+  <si>
     <t>begin_repeat</t>
   </si>
   <si>
-    <t>voter_repeat</t>
-  </si>
-  <si>
     <t>Voter Survey</t>
   </si>
   <si>
     <t>मतदाता सर्वेक्षण</t>
   </si>
   <si>
+    <t>enum_instruction_start</t>
+  </si>
+  <si>
     <t>note</t>
   </si>
   <si>
-    <t>enum_instruction_start</t>
-  </si>
-  <si>
     <t>[Enumerator Instruction]&lt;br/&gt;&lt;br/&gt;1. Tap the &lt;b&gt;Save Icon (diskette)&lt;/b&gt; at the top of the screen to save the form progress.&lt;br/&gt;2. Hand the device over to the next voter to capture their details.</t>
   </si>
   <si>
     <t>[साक्षात्कारकर्ता निर्देश]&lt;br/&gt;&lt;br/&gt;1. फॉर्म की प्रगति को सहेजने के लिए स्क्रीन के शीर्ष पर स्थित &lt;b&gt;सेव आइकन (डिस्केट)&lt;/b&gt; पर टैप करें.&lt;br/&gt;2. अगले मतदाता के विवरण दर्ज करने के लिए उपकरण उन्हें सौंपें.</t>
   </si>
   <si>
+    <t>gender</t>
+  </si>
+  <si>
     <t>select_one gender_list</t>
   </si>
   <si>
-    <t>gender</t>
-  </si>
-  <si>
     <t>Gender</t>
   </si>
   <si>
     <t>लिंग</t>
   </si>
   <si>
+    <t>religion</t>
+  </si>
+  <si>
     <t>select_one religion_list</t>
   </si>
   <si>
-    <t>religion</t>
-  </si>
-  <si>
     <t>Religion</t>
   </si>
   <si>
@@ -216,15 +212,33 @@
     <t>Other Religion (Please specify)</t>
   </si>
   <si>
+    <t>अन्य धर्म (कृपया स्पष्ट करें)</t>
+  </si>
+  <si>
     <t>${religion} = 'other'</t>
   </si>
   <si>
+    <t>voter_id</t>
+  </si>
+  <si>
+    <t>concat(${state}, 'V', once(int(random() * 9000000) + 1000000))</t>
+  </si>
+  <si>
+    <t>show_voter_id</t>
+  </si>
+  <si>
+    <t>Your unique Voter ID (EPIC Number) is: &lt;b&gt;${voter_id}&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>आपका विशिष्ट मतदाता पहचान पत्र (ईपीआईसी संख्या) है: &lt;b&gt;${voter_id}&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>party_vote</t>
+  </si>
+  <si>
     <t>select_one party_list</t>
   </si>
   <si>
-    <t>party_vote</t>
-  </si>
-  <si>
     <t>Cast Your Vote (EVM)</t>
   </si>
   <si>
@@ -261,12 +275,12 @@
     <t>साक्षात्कारकर्ता की टिप्पणी</t>
   </si>
   <si>
+    <t>location</t>
+  </si>
+  <si>
     <t>geopoint</t>
   </si>
   <si>
-    <t>location</t>
-  </si>
-  <si>
     <t>GPS Location</t>
   </si>
   <si>
@@ -342,6 +356,15 @@
     <t>दक्षिण दिल्ली</t>
   </si>
   <si>
+    <t>NDD</t>
+  </si>
+  <si>
+    <t>North Delhi</t>
+  </si>
+  <si>
+    <t>उत्तर दिल्ली</t>
+  </si>
+  <si>
     <t>MC</t>
   </si>
   <si>
@@ -360,6 +383,15 @@
     <t>पुणे</t>
   </si>
   <si>
+    <t>NG</t>
+  </si>
+  <si>
+    <t>Nagpur</t>
+  </si>
+  <si>
+    <t>नागपुर</t>
+  </si>
+  <si>
     <t>LK</t>
   </si>
   <si>
@@ -378,24 +410,6 @@
     <t>वाराणसी</t>
   </si>
   <si>
-    <t>NDD</t>
-  </si>
-  <si>
-    <t>North Delhi</t>
-  </si>
-  <si>
-    <t>उत्तर दिल्ली</t>
-  </si>
-  <si>
-    <t>NG</t>
-  </si>
-  <si>
-    <t>Nagpur</t>
-  </si>
-  <si>
-    <t>नागपुर</t>
-  </si>
-  <si>
     <t>GK</t>
   </si>
   <si>
@@ -696,34 +710,31 @@
     <t>nota.png</t>
   </si>
   <si>
+    <t>form_id</t>
+  </si>
+  <si>
+    <t>form_title</t>
+  </si>
+  <si>
+    <t>default_language</t>
+  </si>
+  <si>
     <t>version</t>
   </si>
   <si>
-    <t>default_language</t>
+    <t>public_key</t>
+  </si>
+  <si>
+    <t>submission_url</t>
   </si>
   <si>
     <t>all_voting_form_repeat_v1</t>
   </si>
   <si>
+    <t>All Voting Form (Repeat)</t>
+  </si>
+  <si>
     <t>English (en)</t>
-  </si>
-  <si>
-    <t>form_id</t>
-  </si>
-  <si>
-    <t>form_title</t>
-  </si>
-  <si>
-    <t>All Voting Form (Repeat)</t>
-  </si>
-  <si>
-    <t>public_key</t>
-  </si>
-  <si>
-    <t>submission_url</t>
-  </si>
-  <si>
-    <t>अन्य धर्म (कृपया स्पष्ट करें)</t>
   </si>
 </sst>
 </file>
@@ -1103,7 +1114,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="13.109375" customWidth="1"/>
@@ -1112,10 +1123,10 @@
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1187,10 +1198,10 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
         <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
       </c>
       <c r="G7" t="s">
         <v>18</v>
@@ -1204,7 +1215,7 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
         <v>18</v>
@@ -1215,10 +1226,10 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
         <v>23</v>
-      </c>
-      <c r="B9" t="s">
-        <v>22</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
@@ -1232,10 +1243,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
         <v>28</v>
-      </c>
-      <c r="B10" t="s">
-        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>29</v>
@@ -1252,10 +1263,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
         <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
       </c>
       <c r="C11" t="s">
         <v>34</v>
@@ -1272,10 +1283,10 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
         <v>38</v>
-      </c>
-      <c r="B12" t="s">
-        <v>37</v>
       </c>
       <c r="C12" t="s">
         <v>39</v>
@@ -1289,10 +1300,10 @@
     </row>
     <row r="13" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>43</v>
@@ -1306,10 +1317,10 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" t="s">
         <v>46</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
       </c>
       <c r="C14" t="s">
         <v>47</v>
@@ -1323,10 +1334,10 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" t="s">
         <v>50</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
@@ -1340,10 +1351,10 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
         <v>54</v>
-      </c>
-      <c r="B16" t="s">
-        <v>53</v>
       </c>
       <c r="C16" t="s">
         <v>55</v>
@@ -1360,19 +1371,19 @@
         <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
         <v>58</v>
       </c>
       <c r="D17" t="s">
-        <v>228</v>
+        <v>59</v>
       </c>
       <c r="G17" t="s">
         <v>26</v>
       </c>
       <c r="J17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
@@ -1380,92 +1391,117 @@
         <v>61</v>
       </c>
       <c r="B18" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" t="s">
         <v>62</v>
-      </c>
-      <c r="D18" t="s">
-        <v>63</v>
-      </c>
-      <c r="E18" t="s">
-        <v>64</v>
-      </c>
-      <c r="F18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G18" t="s">
-        <v>26</v>
-      </c>
-      <c r="K18" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" t="s">
         <v>67</v>
       </c>
-      <c r="B19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="C20" t="s">
         <v>68</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D20" t="s">
         <v>69</v>
       </c>
-      <c r="G19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="4" t="s">
+      <c r="E20" t="s">
         <v>70</v>
+      </c>
+      <c r="F20" t="s">
+        <v>71</v>
+      </c>
+      <c r="G20" t="s">
+        <v>26</v>
+      </c>
+      <c r="K20" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G21" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" t="s">
-        <v>74</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="B22" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D22" t="s">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>77</v>
       </c>
-      <c r="E22" t="s">
+      <c r="B23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" t="s">
         <v>78</v>
       </c>
-      <c r="F22" t="s">
+      <c r="D23" t="s">
         <v>79</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" t="s">
+        <v>85</v>
+      </c>
+      <c r="G24" t="s">
         <v>26</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -1485,10 +1521,10 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -1497,145 +1533,145 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E6" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C7" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" t="s">
         <v>94</v>
-      </c>
-      <c r="B8" t="s">
-        <v>101</v>
-      </c>
-      <c r="C8" t="s">
-        <v>102</v>
-      </c>
-      <c r="D8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E8" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E9" t="s">
         <v>94</v>
-      </c>
-      <c r="B9" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" t="s">
-        <v>105</v>
-      </c>
-      <c r="D9" t="s">
-        <v>106</v>
-      </c>
-      <c r="E9" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B10" t="s">
         <v>116</v>
@@ -1647,304 +1683,304 @@
         <v>118</v>
       </c>
       <c r="E10" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D11" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="E11" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D12" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="E12" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B13" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C13" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D13" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="E13" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B14" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D14" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E14" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B15" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C15" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D15" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E15" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B16" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D16" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E16" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B17" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C17" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D17" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E17" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B18" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C18" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D18" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E18" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B19" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C19" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D19" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E19" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B20" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C20" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="E20" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B21" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C21" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D21" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="E21" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B22" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D22" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="E22" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B23" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C23" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D23" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E23" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>128</v>
+      </c>
+      <c r="B24" t="s">
+        <v>151</v>
+      </c>
+      <c r="C24" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" t="s">
+        <v>124</v>
+      </c>
+      <c r="E24" t="s">
         <v>122</v>
-      </c>
-      <c r="B24" t="s">
-        <v>145</v>
-      </c>
-      <c r="C24" t="s">
-        <v>111</v>
-      </c>
-      <c r="D24" t="s">
-        <v>112</v>
-      </c>
-      <c r="E24" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>128</v>
+      </c>
+      <c r="B25" t="s">
+        <v>152</v>
+      </c>
+      <c r="C25" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" t="s">
+        <v>154</v>
+      </c>
+      <c r="E25" t="s">
         <v>122</v>
-      </c>
-      <c r="B25" t="s">
-        <v>146</v>
-      </c>
-      <c r="C25" t="s">
-        <v>147</v>
-      </c>
-      <c r="D25" t="s">
-        <v>148</v>
-      </c>
-      <c r="E25" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B26" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C26" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D26" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E26" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C27" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D27" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E27" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C28" t="s">
         <v>117</v>
@@ -1958,16 +1994,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C29" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D29" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="E29" t="s">
         <v>116</v>
@@ -1975,321 +2011,321 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B30" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C30" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D30" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="E30" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B31" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C31" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="D31" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E31" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B32" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C32" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="D32" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B33" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C33" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="D33" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B34" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="C34" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="D34" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B35" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C35" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D35" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B36" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C36" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D36" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B37" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C37" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D37" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B38" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C38" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D38" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B39" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C39" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="D39" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B40" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C40" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="D40" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B41" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="C41" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="D41" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B42" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C42" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="D42" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="F42" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="G42" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B43" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="C43" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D43" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="F43" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="G43" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B44" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C44" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D44" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="F44" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="G44" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B45" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C45" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="D45" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="F45" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="G45" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B46" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C46" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D46" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="F46" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G46" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B47" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C47" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D47" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="F47" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="G47" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B48" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="C48" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="D48" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="F48" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="G48" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -2308,41 +2344,41 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="B2" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="C2" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="D2" t="str">
         <f ca="1">TEXT(YEAR(NOW())-2000, "00") &amp; TEXT(MONTH(NOW()), "00") &amp; TEXT(DAY(NOW()), "00") &amp; TEXT(HOUR(NOW()), "00") &amp; TEXT(MINUTE(NOW()), "00")</f>
-        <v>2607082208</v>
+        <v>2607082325</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>